<commit_message>
feat(listener): capture screenshots on test success and failure
</commit_message>
<xml_diff>
--- a/rubeus-qa-tests/reports/QA_Report.xlsx
+++ b/rubeus-qa-tests/reports/QA_Report.xlsx
@@ -53,7 +53,7 @@
     <t>Certification page loaded successfully with correct URL, title and content.</t>
   </si>
   <si>
-    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\certificacao_success_validateCertificacaoPage_success_2026-03-02_16-23-23.png</t>
+    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\certificacao_success_validateCertificacaoPage_success_2026-03-02_16-48-11.png</t>
   </si>
   <si>
     <t>Site</t>
@@ -62,7 +62,7 @@
     <t>Site page loaded successfully with correct URL, title and content.</t>
   </si>
   <si>
-    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\site_success_validateSitePage_success_2026-03-02_16-23-32.png</t>
+    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\site_success_validateSitePage_success_2026-03-02_16-48-19.png</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
fix(BaseTest): resolve screenshot error after driver quit
</commit_message>
<xml_diff>
--- a/rubeus-qa-tests/reports/QA_Report.xlsx
+++ b/rubeus-qa-tests/reports/QA_Report.xlsx
@@ -53,7 +53,7 @@
     <t>Certification page loaded successfully with correct URL, title and content.</t>
   </si>
   <si>
-    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\certificacao_success_validateCertificacaoPage_success_2026-03-02_16-48-11.png</t>
+    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\certificacao_success_validateCertificacaoPage_success_2026-03-02_17-05-28.png</t>
   </si>
   <si>
     <t>Site</t>
@@ -62,7 +62,7 @@
     <t>Site page loaded successfully with correct URL, title and content.</t>
   </si>
   <si>
-    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\site_success_validateSitePage_success_2026-03-02_16-48-19.png</t>
+    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\site_success_validateSitePage_success_2026-03-02_17-05-38.png</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
refactor(TestUtils): remove duplicate waitForPageLoad from takeScreenshot
</commit_message>
<xml_diff>
--- a/rubeus-qa-tests/reports/QA_Report.xlsx
+++ b/rubeus-qa-tests/reports/QA_Report.xlsx
@@ -53,7 +53,7 @@
     <t>Certification page loaded successfully with correct URL, title and content.</t>
   </si>
   <si>
-    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\certificacao_success_validateCertificacaoPage_success_2026-03-02_17-05-28.png</t>
+    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\certificacao_success_validateCertificacaoPage_success_2026-03-02_17-11-56.png</t>
   </si>
   <si>
     <t>Site</t>
@@ -62,7 +62,7 @@
     <t>Site page loaded successfully with correct URL, title and content.</t>
   </si>
   <si>
-    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\site_success_validateSitePage_success_2026-03-02_17-05-38.png</t>
+    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\site_success_validateSitePage_success_2026-03-02_17-12-06.png</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
refactor: pom for include reports
</commit_message>
<xml_diff>
--- a/rubeus-qa-tests/reports/QA_Report.xlsx
+++ b/rubeus-qa-tests/reports/QA_Report.xlsx
@@ -53,7 +53,7 @@
     <t>Certification page loaded successfully with correct URL, title and content.</t>
   </si>
   <si>
-    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\certificacao_success_validateCertificacaoPage_success_2026-03-02_17-11-56.png</t>
+    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\certificacao_success_validateCertificacaoPage_success_2026-03-02_17-28-44.png</t>
   </si>
   <si>
     <t>Site</t>
@@ -62,7 +62,7 @@
     <t>Site page loaded successfully with correct URL, title and content.</t>
   </si>
   <si>
-    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\site_success_validateSitePage_success_2026-03-02_17-12-06.png</t>
+    <t>C:\Users\Alexander\Downloads\AECA\node_sistemas\QA_Analyst\rubeus-qa-tests\screenshots\2026-03-02\site_success_validateSitePage_success_2026-03-02_17-28-56.png</t>
   </si>
 </sst>
 </file>

</xml_diff>